<commit_message>
Expand ROP catalog to 60 raw materials
</commit_message>
<xml_diff>
--- a/sample_data/MRP_full.xlsx
+++ b/sample_data/MRP_full.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="128">
   <si>
     <t>Row Label</t>
   </si>
@@ -64,6 +64,150 @@
     <t>RM-012</t>
   </si>
   <si>
+    <t>RM-013</t>
+  </si>
+  <si>
+    <t>RM-014</t>
+  </si>
+  <si>
+    <t>RM-015</t>
+  </si>
+  <si>
+    <t>RM-016</t>
+  </si>
+  <si>
+    <t>RM-017</t>
+  </si>
+  <si>
+    <t>RM-018</t>
+  </si>
+  <si>
+    <t>RM-019</t>
+  </si>
+  <si>
+    <t>RM-020</t>
+  </si>
+  <si>
+    <t>RM-021</t>
+  </si>
+  <si>
+    <t>RM-022</t>
+  </si>
+  <si>
+    <t>RM-023</t>
+  </si>
+  <si>
+    <t>RM-024</t>
+  </si>
+  <si>
+    <t>RM-025</t>
+  </si>
+  <si>
+    <t>RM-026</t>
+  </si>
+  <si>
+    <t>RM-027</t>
+  </si>
+  <si>
+    <t>RM-028</t>
+  </si>
+  <si>
+    <t>RM-029</t>
+  </si>
+  <si>
+    <t>RM-030</t>
+  </si>
+  <si>
+    <t>RM-031</t>
+  </si>
+  <si>
+    <t>RM-032</t>
+  </si>
+  <si>
+    <t>RM-033</t>
+  </si>
+  <si>
+    <t>RM-034</t>
+  </si>
+  <si>
+    <t>RM-035</t>
+  </si>
+  <si>
+    <t>RM-036</t>
+  </si>
+  <si>
+    <t>RM-037</t>
+  </si>
+  <si>
+    <t>RM-038</t>
+  </si>
+  <si>
+    <t>RM-039</t>
+  </si>
+  <si>
+    <t>RM-040</t>
+  </si>
+  <si>
+    <t>RM-041</t>
+  </si>
+  <si>
+    <t>RM-042</t>
+  </si>
+  <si>
+    <t>RM-043</t>
+  </si>
+  <si>
+    <t>RM-044</t>
+  </si>
+  <si>
+    <t>RM-045</t>
+  </si>
+  <si>
+    <t>RM-046</t>
+  </si>
+  <si>
+    <t>RM-047</t>
+  </si>
+  <si>
+    <t>RM-048</t>
+  </si>
+  <si>
+    <t>RM-049</t>
+  </si>
+  <si>
+    <t>RM-050</t>
+  </si>
+  <si>
+    <t>RM-051</t>
+  </si>
+  <si>
+    <t>RM-052</t>
+  </si>
+  <si>
+    <t>RM-053</t>
+  </si>
+  <si>
+    <t>RM-054</t>
+  </si>
+  <si>
+    <t>RM-055</t>
+  </si>
+  <si>
+    <t>RM-056</t>
+  </si>
+  <si>
+    <t>RM-057</t>
+  </si>
+  <si>
+    <t>RM-058</t>
+  </si>
+  <si>
+    <t>RM-059</t>
+  </si>
+  <si>
+    <t>RM-060</t>
+  </si>
+  <si>
     <t>Wheat Flour</t>
   </si>
   <si>
@@ -98,6 +242,150 @@
   </si>
   <si>
     <t>Lemon Extract</t>
+  </si>
+  <si>
+    <t>Rye Flour</t>
+  </si>
+  <si>
+    <t>Whole Wheat Flour</t>
+  </si>
+  <si>
+    <t>Cornflour</t>
+  </si>
+  <si>
+    <t>Oat Flour</t>
+  </si>
+  <si>
+    <t>Almond Flour</t>
+  </si>
+  <si>
+    <t>Rice Flour</t>
+  </si>
+  <si>
+    <t>Semolina</t>
+  </si>
+  <si>
+    <t>Brown Sugar</t>
+  </si>
+  <si>
+    <t>Caster Sugar</t>
+  </si>
+  <si>
+    <t>Honey</t>
+  </si>
+  <si>
+    <t>Golden Syrup</t>
+  </si>
+  <si>
+    <t>Maple Syrup</t>
+  </si>
+  <si>
+    <t>Glucose Syrup</t>
+  </si>
+  <si>
+    <t>Molasses</t>
+  </si>
+  <si>
+    <t>Demerara Sugar</t>
+  </si>
+  <si>
+    <t>Vegetable Oil</t>
+  </si>
+  <si>
+    <t>Sunflower Oil</t>
+  </si>
+  <si>
+    <t>Olive Oil</t>
+  </si>
+  <si>
+    <t>Shortening</t>
+  </si>
+  <si>
+    <t>Ghee</t>
+  </si>
+  <si>
+    <t>Cream Cheese</t>
+  </si>
+  <si>
+    <t>Sour Cream</t>
+  </si>
+  <si>
+    <t>Condensed Milk</t>
+  </si>
+  <si>
+    <t>Buttermilk</t>
+  </si>
+  <si>
+    <t>Fresh Cream</t>
+  </si>
+  <si>
+    <t>Yogurt</t>
+  </si>
+  <si>
+    <t>Yeast</t>
+  </si>
+  <si>
+    <t>Cream of Tartar</t>
+  </si>
+  <si>
+    <t>Cinnamon</t>
+  </si>
+  <si>
+    <t>Nutmeg</t>
+  </si>
+  <si>
+    <t>Cardamom</t>
+  </si>
+  <si>
+    <t>Ginger Powder</t>
+  </si>
+  <si>
+    <t>Coffee Extract</t>
+  </si>
+  <si>
+    <t>Vanilla Bean Paste</t>
+  </si>
+  <si>
+    <t>Almond Essence</t>
+  </si>
+  <si>
+    <t>Cocoa Butter</t>
+  </si>
+  <si>
+    <t>Dark Chocolate</t>
+  </si>
+  <si>
+    <t>White Chocolate</t>
+  </si>
+  <si>
+    <t>Chocolate Chips</t>
+  </si>
+  <si>
+    <t>Caramel</t>
+  </si>
+  <si>
+    <t>Hazelnut Spread</t>
+  </si>
+  <si>
+    <t>Raspberry Jam</t>
+  </si>
+  <si>
+    <t>Blueberry Jam</t>
+  </si>
+  <si>
+    <t>Mango Puree</t>
+  </si>
+  <si>
+    <t>Coconut Flakes</t>
+  </si>
+  <si>
+    <t>Chopped Nuts</t>
+  </si>
+  <si>
+    <t>Peanut Butter</t>
+  </si>
+  <si>
+    <t>Lemon Curd</t>
   </si>
   <si>
     <t>kg</t>
@@ -441,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -463,13 +751,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="C2">
         <v>420</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -477,13 +765,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="C3">
         <v>300</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -491,13 +779,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="C4">
         <v>240</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -505,13 +793,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="C5">
         <v>4200</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -519,13 +807,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -533,13 +821,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C7">
         <v>90</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -547,13 +835,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="C8">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -561,13 +849,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="C9">
         <v>900</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -575,13 +863,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="C10">
         <v>160</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -589,13 +877,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C11">
         <v>110</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -603,13 +891,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="C12">
         <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -617,13 +905,685 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="C13">
         <v>300</v>
       </c>
       <c r="D13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14">
+        <v>180</v>
+      </c>
+      <c r="D14" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15">
+        <v>210</v>
+      </c>
+      <c r="D15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17">
+        <v>120</v>
+      </c>
+      <c r="D17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18">
+        <v>160</v>
+      </c>
+      <c r="D18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19">
+        <v>85</v>
+      </c>
+      <c r="D19" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20">
+        <v>70</v>
+      </c>
+      <c r="D20" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21">
+        <v>240</v>
+      </c>
+      <c r="D21" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22">
+        <v>320</v>
+      </c>
+      <c r="D22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23">
+        <v>65</v>
+      </c>
+      <c r="D23" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24">
+        <v>90</v>
+      </c>
+      <c r="D24" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25">
+        <v>40</v>
+      </c>
+      <c r="D25" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26">
+        <v>75</v>
+      </c>
+      <c r="D26" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27">
+        <v>25</v>
+      </c>
+      <c r="D27" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28">
+        <v>110</v>
+      </c>
+      <c r="D28" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
         <v>31</v>
+      </c>
+      <c r="B29" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29">
+        <v>120</v>
+      </c>
+      <c r="D29" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30">
+        <v>45</v>
+      </c>
+      <c r="D30" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+      <c r="D31" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32">
+        <v>60</v>
+      </c>
+      <c r="D32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33">
+        <v>35</v>
+      </c>
+      <c r="D33" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34">
+        <v>140</v>
+      </c>
+      <c r="D34" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35">
+        <v>80</v>
+      </c>
+      <c r="D35" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36">
+        <v>55</v>
+      </c>
+      <c r="D36" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37">
+        <v>70</v>
+      </c>
+      <c r="D37" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38">
+        <v>200</v>
+      </c>
+      <c r="D38" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39">
+        <v>90</v>
+      </c>
+      <c r="D39" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41">
+        <v>6</v>
+      </c>
+      <c r="D41" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42">
+        <v>5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" t="s">
+        <v>105</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47">
+        <v>6</v>
+      </c>
+      <c r="D47" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" t="s">
+        <v>110</v>
+      </c>
+      <c r="C48">
+        <v>3</v>
+      </c>
+      <c r="D48" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" t="s">
+        <v>111</v>
+      </c>
+      <c r="C49">
+        <v>12</v>
+      </c>
+      <c r="D49" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" t="s">
+        <v>112</v>
+      </c>
+      <c r="C50">
+        <v>85</v>
+      </c>
+      <c r="D50" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51">
+        <v>75</v>
+      </c>
+      <c r="D51" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C52">
+        <v>95</v>
+      </c>
+      <c r="D52" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" t="s">
+        <v>115</v>
+      </c>
+      <c r="C53">
+        <v>60</v>
+      </c>
+      <c r="D53" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" t="s">
+        <v>116</v>
+      </c>
+      <c r="C54">
+        <v>70</v>
+      </c>
+      <c r="D54" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" t="s">
+        <v>117</v>
+      </c>
+      <c r="C55">
+        <v>50</v>
+      </c>
+      <c r="D55" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" t="s">
+        <v>118</v>
+      </c>
+      <c r="C56">
+        <v>45</v>
+      </c>
+      <c r="D56" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" t="s">
+        <v>119</v>
+      </c>
+      <c r="C57">
+        <v>40</v>
+      </c>
+      <c r="D57" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" t="s">
+        <v>120</v>
+      </c>
+      <c r="C58">
+        <v>35</v>
+      </c>
+      <c r="D58" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" t="s">
+        <v>121</v>
+      </c>
+      <c r="C59">
+        <v>55</v>
+      </c>
+      <c r="D59" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" t="s">
+        <v>122</v>
+      </c>
+      <c r="C60">
+        <v>40</v>
+      </c>
+      <c r="D60" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" t="s">
+        <v>123</v>
+      </c>
+      <c r="C61">
+        <v>25</v>
+      </c>
+      <c r="D61" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>